<commit_message>
Update cyber incident intelligence
</commit_message>
<xml_diff>
--- a/japan_cyber_incidents_1month.xlsx
+++ b/japan_cyber_incidents_1month.xlsx
@@ -4988,7 +4988,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTE94V2trWWZwRDhaOEo3ajV6cWtwVktyaGhuMFJLb1R0RDJBeW1FQzhvek4xN1libEZTbFVpcERRYmpVUmEyN0JXRkdiLXQzd3pfUHdNRGJOQUxERjlvNVlIRzU1ZS0ycGJDbXJILUMyb9IBdEFVX3lxTE80RFY0X1VyNVh1al9tTWVzc3pHLW9PWDk0SXdoSWNxTHZNenh6OUwweTh0Wk9SZGl0ZENodmVDVEpLdFoxR3h6TlQyVGU2NjNsVjBwT0wwRXhBblRUMTN3aVA1UUpWYTU1Tzc0OG9zZF9pWDM1?oc=5 / https://news.google.com/rss/articles/CBMid0FVX3lxTFA2TF9lSXVjc0V3RFgtVGdpc0lVczZZa3Z0MlkzWXNJczhicV9adTQ4T2VKeEFFR3ZTa3FNQkFrRVBHWTRVc0dMV3ZwNG1MV2lod0kyZXo3eU9iVUdTRnRhU1BlbUNzSWJwYnhJalg4S05FT2hYVENV0gF8QVVfeXFMUHdkZGMzS00zZXJRa1FhemRWLU9SS3ZWejdjdmgyaWNJb0tCazBjenNPQllFOWkwbnhwVUlXMjRMS1E1LWhKMUtWWm5XYkotZEQ3WlRnU1VsdDRGUV9FbVBMRnpmUlRXbkNOb1doSF9vdDBoaERiWmdhejJwSQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTE94V2trWWZwRDhaOEo3ajV6cWtwVktyaGhuMFJLb1R0RDJBeW1FQzhvek4xN1libEZTbFVpcERRYmpVUmEyN0JXRkdiLXQzd3pfUHdNRGJOQUxERjlvNVlIRzU1ZS0ycGJDbXJILUMyb9IBdEFVX3lxTE80RFY0X1VyNVh1al9tTWVzc3pHLW9PWDk0SXdoSWNxTHZNenh6OUwweTh0Wk9SZGl0ZENodmVDVEpLdFoxR3h6TlQyVGU2NjNsVjBwT0wwRXhBblRUMTN3aVA1UUpWYTU1Tzc0OG9zZF9pWDM1?oc=5 / https://news.google.com/rss/articles/CBMif0FVX3lxTE1Ub0xVTmY1N1ZxUWstRTZLZmhKMjJuQ0gyVWVjdUJmc0xmSk5FbTFGVUxMLUl6bnhGZmltWWtzNlhEZmJtWmFhS2VhX3MxbmNFVkJzTGNZRWpfRUhEaGJ1VElaczFzcUhGWW8teWVhNDdoMkg3ZG8xRWMyTVlMMVE?oc=5 / https://news.google.com/rss/articles/CBMid0FVX3lxTFA2TF9lSXVjc0V3RFgtVGdpc0lVczZZa3Z0MlkzWXNJczhicV9adTQ4T2VKeEFFR3ZTa3FNQkFrRVBHWTRVc0dMV3ZwNG1MV2lod0kyZXo3eU9iVUdTRnRhU1BlbUNzSWJwYnhJalg4S05FT2hYVENV0gF8QVVfeXFMUHdkZGMzS00zZXJRa1FhemRWLU9SS3ZWejdjdmgyaWNJb0tCazBjenNPQllFOWkwbnhwVUlXMjRMS1E1LWhKMUtWWm5XYkotZEQ3WlRnU1VsdDRGUV9FbVBMRnpmUlRXbkNOb1doSF9vdDBoaERiWmdhejJwSQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -12647,7 +12647,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-07T00:40:38.339605+00:00</t>
+          <t>2026-10-07T00:41:24.358149+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>